<commit_message>
Add ChatGPT's Resilient City design as a fifth city in the comparison
Folds chat-gpt-code/resilient-city into the sandbox on the same terms as
the four Claude-model designs:

- 5th entry in data/normalized_cities.json (49 figures, same schema; 12
  marked MISSING — no seismic magnitude, no soft-storey ban, no tsunami
  design height, etc. — none inferred)
- genResilientCity() renders its 5x5 square grid of 2 km districts
  (distinct from the four hex/ring forms) and simulates fire/flood/quake
  + population like the others; gas retained (auto-isolated) so it keeps
  post-quake ignition risk, unlike Meridian-F
- Compare view, xlsx and README updated to five cities; crime-metric and
  other comparability warnings extended to include it

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KUZt98FSRwyFQ7Jjz2QHZ9
</commit_message>
<xml_diff>
--- a/city_comparison.xlsx
+++ b/city_comparison.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +61,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00D55181"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -90,7 +94,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -120,6 +124,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="009085E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D55181"/>
       </patternFill>
     </fill>
     <fill>
@@ -159,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,8 +190,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -198,18 +210,21 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,13 +234,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -328,6 +344,11 @@
         <t>source: masterplan §1</t>
       </text>
     </comment>
+    <comment ref="F3" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §1</t>
+      </text>
+    </comment>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan.md header
@@ -349,6 +370,11 @@
         <t>source: masterplan §1</t>
       </text>
     </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §1 (10×10 km)</t>
+      </text>
+    </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>source: 520,000 / 1,965 km2
@@ -371,6 +397,11 @@
         <t>source: masterplan §1</t>
       </text>
     </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §2.3</t>
+      </text>
+    </comment>
     <comment ref="C6" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4
@@ -388,6 +419,11 @@
         <t>source: masterplan §1 ('the only form that has repeatedly delivered &gt;30,000/km2 net')</t>
       </text>
     </comment>
+    <comment ref="F6" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §2.3</t>
+      </text>
+    </comment>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
         <t>source: 25-150 km annulus stated as extractive hinterland; area = pi*(150^2-25^2)
@@ -409,6 +445,11 @@
         <t>source: masterplan §1, §3</t>
       </text>
     </comment>
+    <comment ref="F7" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §1, §4.2</t>
+      </text>
+    </comment>
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §1.1</t>
@@ -429,6 +470,11 @@
         <t>source: masterplan §1</t>
       </text>
     </comment>
+    <comment ref="F8" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §2.3</t>
+      </text>
+    </comment>
     <comment ref="B9" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §2.1</t>
@@ -447,6 +493,11 @@
     <comment ref="E9" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §2</t>
+      </text>
+    </comment>
+    <comment ref="F9" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.2, §4.5</t>
       </text>
     </comment>
     <comment ref="E10" authorId="0" shapeId="0">
@@ -470,6 +521,12 @@
         <t>source: masterplan §2</t>
       </text>
     </comment>
+    <comment ref="F12" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §1, §3.2
+note: unlike Meridian-F's outright gas ban, gas is present but auto-isolated — some post-quake ignition risk retained</t>
+      </text>
+    </comment>
     <comment ref="B14" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §2.1</t>
@@ -491,6 +548,12 @@
         <t>source: masterplan §2</t>
       </text>
     </comment>
+    <comment ref="F14" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.2
+note: framework stated but NO magnitude number (region-tuned) — sim assumes generic M8.0 MCE, flagged</t>
+      </text>
+    </comment>
     <comment ref="B15" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §2.1
@@ -512,6 +575,11 @@
         <t>source: masterplan §2</t>
       </text>
     </comment>
+    <comment ref="F15" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.2</t>
+      </text>
+    </comment>
     <comment ref="C16" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §2.1</t>
@@ -562,6 +630,11 @@
         <t>source: masterplan §2</t>
       </text>
     </comment>
+    <comment ref="F20" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.3</t>
+      </text>
+    </comment>
     <comment ref="C21" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §2.2</t>
@@ -575,6 +648,11 @@
     <comment ref="E21" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §1, §2</t>
+      </text>
+    </comment>
+    <comment ref="F21" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.1, §3.3</t>
       </text>
     </comment>
     <comment ref="B22" authorId="0" shapeId="0">
@@ -593,6 +671,11 @@
         <t>source: masterplan §1, §7</t>
       </text>
     </comment>
+    <comment ref="F22" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.5, §4.3</t>
+      </text>
+    </comment>
     <comment ref="B23" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §2.3</t>
@@ -614,6 +697,12 @@
         <t>source: masterplan §2 cyclonic module</t>
       </text>
     </comment>
+    <comment ref="F23" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.4
+note: no single design wind speed number</t>
+      </text>
+    </comment>
     <comment ref="B25" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4.1
@@ -638,6 +727,12 @@
 note: micro-stations on ~1.4 km triangular lattice; cross-trained fire/EMS/community-police crews of 6-8; base-isolated, solar+battery islanded</t>
       </text>
     </comment>
+    <comment ref="F25" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §2.1, §6.1
+note: one combined fire/medical/rescue station at every 2×2 km district centre</t>
+      </text>
+    </comment>
     <comment ref="B26" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4.1
@@ -662,6 +757,12 @@
 definition: turnout (75 s) + travel at 36 km/h, BFS on 100 m street grid; mean 2.3</t>
       </text>
     </comment>
+    <comment ref="F26" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §6.2
+definition: computed indicative fire arrival: 60 s dispatch + 75 s turnout + expected 1 km Manhattan at 35 km/h; ambulance equivalent 3.46 min</t>
+      </text>
+    </comment>
     <comment ref="B27" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4.1
@@ -680,6 +781,12 @@
 definition: p90 reported, not p95</t>
       </text>
     </comment>
+    <comment ref="F27" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §6.2, §6.3
+note: explicit p95 not printed; the repo's script computes percentiles but the doc reports mean + worst-corner</t>
+      </text>
+    </comment>
     <comment ref="B28" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4.2</t>
@@ -701,6 +808,12 @@
         <t>source: same 33 integrated stations; hospital transport median 3.2 min (4 hospitals)</t>
       </text>
     </comment>
+    <comment ref="F28" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §6.2
+definition: computed: 45 s dispatch + 60 s turnout + 1 km at 35 km/h</t>
+      </text>
+    </comment>
     <comment ref="B29" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4.2</t>
@@ -743,6 +856,11 @@
         <t>source: kōban-model officers embedded in the 33 micro-stations</t>
       </text>
     </comment>
+    <comment ref="F31" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §6.1, §7</t>
+      </text>
+    </comment>
     <comment ref="B32" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4.2</t>
@@ -763,6 +881,11 @@
         <t>source: masterplan §4</t>
       </text>
     </comment>
+    <comment ref="F32" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §2.1, §6.1</t>
+      </text>
+    </comment>
     <comment ref="C33" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §5</t>
@@ -771,6 +894,11 @@
     <comment ref="E33" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4 table</t>
+      </text>
+    </comment>
+    <comment ref="F33" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §6.2, §6.3</t>
       </text>
     </comment>
     <comment ref="B35" authorId="0" shapeId="0">
@@ -796,6 +924,12 @@
 note: plus overall victimisation &lt;50% of host-nation baseline</t>
       </text>
     </comment>
+    <comment ref="F35" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §7.1
+note: multi-metric target: also serious violent victimisation &lt;10/1,000/yr and residential burglary &lt;5/1,000 households/yr</t>
+      </text>
+    </comment>
     <comment ref="B36" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §7.4</t>
@@ -821,6 +955,11 @@
         <t>source: masterplan §6</t>
       </text>
     </comment>
+    <comment ref="F37" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §8</t>
+      </text>
+    </comment>
     <comment ref="B38" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §5.3</t>
@@ -839,6 +978,12 @@
     <comment ref="E40" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §3 (5.5 MWh/person/yr)</t>
+      </text>
+    </comment>
+    <comment ref="F40" authorId="0" shapeId="0">
+      <text>
+        <t>source: 8 TWh/yr demand / 8,760 h
+note: generation sized to ~12 TWh/yr (~1.37 GW avg) for storage losses/reserve</t>
       </text>
     </comment>
     <comment ref="C41" authorId="0" shapeId="0">
@@ -878,6 +1023,12 @@
 note: no % split — firm block sized by geography</t>
       </text>
     </comment>
+    <comment ref="F42" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §4.4
+note: no percentage split — region-tuned</t>
+      </text>
+    </comment>
     <comment ref="B43" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §3.1</t>
@@ -904,6 +1055,12 @@
 note: no multi-day autonomy claim made</t>
       </text>
     </comment>
+    <comment ref="F44" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §3.5, §4.4
+note: 72 h electrical reserve target + 72 h passive building survivability</t>
+      </text>
+    </comment>
     <comment ref="B45" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §3.3
@@ -926,6 +1083,12 @@
         <t>source: 47 Mm3/yr / 365 (130 L/person/day stated); irrigation ~10x municipal in a dry year</t>
       </text>
     </comment>
+    <comment ref="F45" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §4.3
+note: treatment capacity &gt;=200,000 m3/day; industry &amp; agriculture on separate budgets</t>
+      </text>
+    </comment>
     <comment ref="B46" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §3.3</t>
@@ -947,6 +1110,12 @@
 note: no full % split of the stack</t>
       </text>
     </comment>
+    <comment ref="F46" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §4.3
+note: no percentage split; three-network potable/reclaimed/stormwater system</t>
+      </text>
+    </comment>
     <comment ref="B47" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §12</t>
@@ -955,6 +1124,11 @@
     <comment ref="E47" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §7</t>
+      </text>
+    </comment>
+    <comment ref="F47" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §4.3</t>
       </text>
     </comment>
     <comment ref="B48" authorId="0" shapeId="0">
@@ -978,6 +1152,11 @@
         <t>source: masterplan §3</t>
       </text>
     </comment>
+    <comment ref="F48" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §4.2</t>
+      </text>
+    </comment>
     <comment ref="B49" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §3.2</t>
@@ -994,6 +1173,11 @@
         <t>source: masterplan §3, L5</t>
       </text>
     </comment>
+    <comment ref="F49" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §4.2</t>
+      </text>
+    </comment>
     <comment ref="B51" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §7.2</t>
@@ -1014,6 +1198,11 @@
         <t>source: masterplan §5</t>
       </text>
     </comment>
+    <comment ref="F51" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §5.1</t>
+      </text>
+    </comment>
     <comment ref="C52" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §4</t>
@@ -1029,6 +1218,11 @@
         <t>source: masterplan §5</t>
       </text>
     </comment>
+    <comment ref="F52" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §5.1, §5.3</t>
+      </text>
+    </comment>
     <comment ref="B53" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §1.2</t>
@@ -1049,6 +1243,11 @@
         <t>source: masterplan §5</t>
       </text>
     </comment>
+    <comment ref="F53" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §2.2, §5.3</t>
+      </text>
+    </comment>
     <comment ref="C54" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §5, §8</t>
@@ -1057,6 +1256,11 @@
     <comment ref="E54" authorId="0" shapeId="0">
       <text>
         <t>source: masterplan §7</t>
+      </text>
+    </comment>
+    <comment ref="F54" authorId="0" shapeId="0">
+      <text>
+        <t>source: masterplan §4.3, §3.5</t>
       </text>
     </comment>
   </commentList>
@@ -1352,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1513,29 +1717,55 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>chat-gpt-code/resilient-city</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>13 of 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Comparability warnings — read before using any cross-city figure:</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>•  CRIME TARGETS ARE NOT DIRECTLY COMPARABLE: Solaris targets 15 total crimes/100k/yr, Meridian-S targets &lt;150 VIOLENT crimes/100k/yr, CIVITAS and Meridian-F target homicide rates (&lt;1 and &lt;0.5 per 100k/yr respectively). These are different metrics.</t>
-        </is>
-      </c>
-    </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>•  CRIME TARGETS ARE NOT DIRECTLY COMPARABLE: Solaris targets 15 total crimes/100k/yr, Meridian-S targets &lt;150 VIOLENT crimes/100k/yr, and CIVITAS, Meridian-F and Resilient City target homicide rates (&lt;1, &lt;0.5 and &lt;2 per 100k/yr respectively — Resilient City also sets violent-victimisation and burglary sub-targets). These are different metrics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>•  RESPONSE TIMES ARE NOT DIRECTLY COMPARABLE: definitions differ — Solaris reports simulated travel medians, Meridian-S reports travel-to-farthest-resident seconds, CIVITAS reports end-to-end (call to on-scene) including dispatch+turnout, Meridian-F reports turnout+travel. Each figure carries a 'definition' field.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>•  DENSITY BASIS DIFFERS: Solaris's 1,965 km2 footprint includes agricultural rings inside the city boundary; the other three exclude their hinterland from the urban area. Solaris does not state a built-up-only density.</t>
         </is>
@@ -1544,8 +1774,8 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A12:F12"/>
   </mergeCells>
@@ -1559,7 +1789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1567,1367 +1797,1614 @@
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Figure</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>Meridian (Fable)</t>
         </is>
       </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>— Scale &amp; form —</t>
         </is>
       </c>
-      <c r="B2" s="17" t="n"/>
-      <c r="C2" s="17" t="n"/>
-      <c r="D2" s="17" t="n"/>
-      <c r="E2" s="17" t="n"/>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+      <c r="F2" s="19" t="n"/>
     </row>
     <row r="3" ht="46" customHeight="1">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>520000 people</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="21" t="inlineStr">
         <is>
           <t>467031 people</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>250000 people</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>1000000 people</t>
         </is>
       </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>1000000 people</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="46" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Urban area (km²)</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>1965 km2</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>54.0 km2</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>18.0 km2</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>54.5 km2</t>
         </is>
       </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>100 km2</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Gross density (people/km²)</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>265 people/km2</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>8650 people/km2</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>13900 people/km2</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>18300 people/km2</t>
         </is>
       </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>10000 people/km2</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Built-up density (people/km²)</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>MISSING — masterplan gives ring populations and radii but never a built-up density figure</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>22000 people/km2</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>13900 people/km2</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>30000 people/km2 net residential (typology figure)</t>
         </is>
       </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>20000-35000 people/km2 (inhabited mixed-use portions)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Hinterland footprint (km²)</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>68700 km2</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>388 km2 farmland (7.2x city) + 17.8 km2 aquaculture bay</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>244 km2 (217 farm + 27 energy; total region 262 km2, ~9 km radius)</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>1250 km2 (~20 km radius)</t>
         </is>
       </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>4000 km2 (reference; range 3,500-4,500)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Typical building storeys</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>8-35 by ring</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>6-10 (housing); 25-30 landmark towers at district hubs only</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>5-8 perimeter blocks; landmark tower + vertical farms taller</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>6-8 perimeter blocks; 12-20 storey clusters within 400 m of district hubs</t>
         </is>
       </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>6-18 storeys; taller towers exceptional</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Primary building materials</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>CLT or reinforced concrete (ductile detailing)</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>ductile reinforced concrete or mass timber moment frames with shear walls</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>RC/steel ductile frames; CLT mid-rise where forestry supplies; rammed earth/CSEB; geopolymer cement</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>engineered mass timber (CLT) or reinforced concrete, strong-column/weak-beam</t>
         </is>
       </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>ductile reinforced concrete, steel or engineered timber; low-clinker cement, reclaimed aggregate, electric-furnace recycled metal</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Street width (m)</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>MISSING — 'strict building separation distances' asserted in §10.1 but no number anywhere</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>MISSING — cell geometry and 180 m inter-district buffers stated; street cross-sections not</t>
         </is>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>MISSING — block typology described; street cross-sections not dimensioned</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>20 m</t>
         </is>
       </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — superblocks + redundant street grid described; no street cross-section dimension stated</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Building spacing / block grid</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>MISSING — no spacing, setback, or block-grid dimension stated — fire-spread modelling for Solaris is low-confidence</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>180 m green buffers between districts (double as firebreaks); shared green edge around each cell</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="23" t="inlineStr">
         <is>
           <t>MISSING — perimeter-block courtyards implied; no block-grid dimension given</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>~130 m perimeter-block grid, 20 m streets</t>
         </is>
       </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — 2×2 km districts with superblocks and a redundant utility/transit street grid stated, but no block-grid dimension — fire-spread geometry approximated</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Gas grid / ignition source</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>MISSING — post-quake fire ignition source unaddressed (Meridian-F explicitly bans gas; Solaris silent)</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>MISSING — buried utilities stated for wind; gas not addressed</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>none — all-electric city, gas omitted to remove post-quake ignition (Kobe lesson)</t>
         </is>
       </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>mostly electrified (transport/heating/industry); automatic gas &amp; hazardous-process isolation — gas not fully eliminated</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>— Structural resilience —</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="17" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
     </row>
     <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Seismic design basis</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>9.0 Mw</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>M9-class subduction (coastal Pacific-Rim worst case)</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>MCE — Life Safety for residential, Immediate Occupancy for lifelines</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>site MCE, e.g. M8+ subduction or M7 crustal; microzonation &lt;=200 m mandatory before construction</t>
         </is>
       </c>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>site-specific performance-based: Immediate Occupancy (frequent), Repairable (design-basis), No Collapse (MCE), No Progressive Collapse (beyond-design)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="46" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Base isolation scope</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>all buildings &gt;=8 storeys</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>critical/hub buildings only (hospitals, schools, fire/EMS stations, civic core)</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>hospital, 7 emergency hubs, civic tower, evacuation towers</t>
         </is>
       </c>
-      <c r="E15" s="19" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>hospitals, all 33 micro-stations, water/energy control nodes, district civic halls</t>
         </is>
       </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>hospitals, control centres, water plants, refuge buildings, and selected residential/civic buildings</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="46" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Soft-storey ban</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>MISSING — not addressed (waterfront buildings deliberately have open lower storeys for tsunami)</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="23" t="inlineStr">
         <is>
           <t>MISSING — strong-column/weak-beam stated; explicit soft-storey prohibition not stated (seaward pilotis blocks are deliberately open-ground)</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — capacity design + strong-column/weak-beam stated, but no explicit soft-storey prohibition (contrast Meridian-F/S which ban it outright)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="46" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Lateral drift capacity (m)</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>1.5 m lateral</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — not reported in source repo</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="46" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Quake survival target (%)</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>99.5 % at 9.0 Mw</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>MISSING — no quantified survival target; qualitative performance goals only</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="23" t="inlineStr">
         <is>
           <t>MISSING — no % survival target; instead a functional target — lattice still serves city with 25% of stations destroyed (computed)</t>
         </is>
       </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — qualitative 'no collapse at MCE / no progressive collapse beyond design'; no % survival figure</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="46" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Tsunami / surge design height (m)</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>15 m</t>
         </is>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>MISSING — refuge storeys 'above the design tsunami height' and high-ground network at +15-20 m stated, but the design wave height itself is never given</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="23" t="inlineStr">
         <is>
           <t>MISSING — layered defence + FEMA P-646 refuges stated; design wave height region-tuned, never numbered</t>
         </is>
       </c>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>15 m (berm at +15 m; habitable floors above +15 m; 1-in-1000-yr design basis)</t>
         </is>
       </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — defence is avoidance (build landward of the site-specific extreme inundation line); the inundation height itself is never numbered</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="46" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Flood defence layers</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>5 m artificial dunes + mangroves + breakwaters; open lower 3 storeys within 2 km of coast; roof evacuation; 2-min sensor warning</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t>dune+mangrove buffer; seawall with retractable surge gate; elevated ring road berm; refuge storey per building; critical services on +15-20 m podium network</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>forested berm + mangroves/dunes; core on raised terp; sacrificial flow-through pilotis on seaward blocks; vertical refuges within 5-min walk</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>living shoreline; +15 m landscape berm; sacrificial 400 m waterfront band (no ground-floor housing); vertical evacuation within 10-min walk; wedges as floodways</t>
         </is>
       </c>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>avoidance-first: uninhabited wetland/dune/floodable-park belt; development landward of extreme inundation line; raised redundant high-ground route; vertical-evacuation structures; breakaway ground-floor walls on edge structures; scour-designed deep foundations; independent-power drainage pumps; local detection</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="46" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Site elevation / terrain data</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>MISSING — no ground elevations, drainage capacities, or inundation map — flood simulation is low-confidence and defence-layer-based only</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>partial — critical podium network at +15-20 m stated; no terrain map</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>partial — 'urban core sits on raised ground (engineered terp)'; no heights given</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>partial — berm +15 m, habitable floors +15 m, wedges as stormwater basins/floodways; no full terrain map</t>
         </is>
       </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t>partial — critical facilities on strongest ground above credible flood levels; raised high-ground evacuation route; no terrain map</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="46" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Stormwater drainage</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>radial canal corridors</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>MISSING — buffers include 'drainage swales' (geometry script) but no capacities</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>looped utilidor network with sectionalising valves (water); stormwater not separately specified</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E22" s="21" t="inlineStr">
         <is>
           <t>stormwater basins in green wedges; rooftop catchment mandated (L19)</t>
         </is>
       </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>dedicated third network for stormwater &amp; flood conveyance; gravity drainage + independent-power pumps; looped water network with district cisterns</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="46" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Wind design</t>
         </is>
       </c>
-      <c r="B23" s="19" t="inlineStr">
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>Category 5 / 250 km/h sustained</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>Category 5-equivalent; Miami-Dade continuous load path; TMD/TLD on landmark towers</t>
         </is>
       </c>
-      <c r="D23" s="19" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>typhoon/hurricane package: aerodynamic massing, continuous load path (Miami-Dade), impact glazing, buried utilities</t>
         </is>
       </c>
-      <c r="E23" s="19" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>250 km/h 3-s gust (Saffir-Simpson 5); Miami-Dade envelope; underground grid; TMD on tall buildings</t>
         </is>
       </c>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t>greater of local code event or site-specific study; continuous load path, impact-rated glazing, hip roofs, refuge rooms; higher importance factor for critical buildings</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>— Emergency response —</t>
         </is>
       </c>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="17" t="n"/>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="17" t="n"/>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Fire stations</t>
         </is>
       </c>
-      <c r="B25" s="19" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="C25" s="20" t="inlineStr">
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>6 district main fire/EMS stations + ~43 cell-hub micro-posts (paramedic e-bike + AED drone)</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E25" s="19" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
+      <c r="F25" s="21" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>Fire response, median (min)</t>
         </is>
       </c>
-      <c r="B26" s="19" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>4.2 min</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C26" s="21" t="inlineStr">
         <is>
           <t>2.0 min</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>3.71 min</t>
         </is>
       </c>
-      <c r="E26" s="19" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>2.4 min</t>
         </is>
       </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>3.96 min</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="46" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Fire response, tail (min)</t>
         </is>
       </c>
-      <c r="B27" s="19" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>5.2 min</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C27" s="23" t="inlineStr">
         <is>
           <t>MISSING — model reports median and zero-points-over-300s, not a p95</t>
         </is>
       </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>4.32 min</t>
         </is>
       </c>
-      <c r="E27" s="19" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>2.8 min (p90; max 3.9)</t>
         </is>
       </c>
+      <c r="F27" s="21" t="inlineStr">
+        <is>
+          <t>7.05 min worst-corner (degraded 25 km/h roads); target 90% &lt;5 min</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="46" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>EMS response, median (min)</t>
         </is>
       </c>
-      <c r="B28" s="19" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>5.1 min</t>
         </is>
       </c>
-      <c r="C28" s="19" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>2.0 min</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>3.71 min</t>
         </is>
       </c>
-      <c r="E28" s="19" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>2.4 min</t>
         </is>
       </c>
+      <c r="F28" s="21" t="inlineStr">
+        <is>
+          <t>3.46 min</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="46" customHeight="1">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>Ambulances</t>
         </is>
       </c>
-      <c r="B29" s="19" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C29" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr">
         <is>
           <t>MISSING — hubs co-locate EMS; vehicle counts not given</t>
         </is>
       </c>
-      <c r="E29" s="19" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — combined stations described; ambulance/vehicle counts not given</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="46" customHeight="1">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>Police response (min)</t>
         </is>
       </c>
-      <c r="B30" s="19" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>8 min</t>
         </is>
       </c>
-      <c r="C30" s="21" t="inlineStr">
+      <c r="C30" s="23" t="inlineStr">
         <is>
           <t>MISSING — policing legitimacy/accountability specified; response times and station counts are not</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>3.71 min (same hubs)</t>
         </is>
       </c>
-      <c r="E30" s="20" t="inlineStr">
+      <c r="E30" s="22" t="inlineStr">
         <is>
           <t>2.4 min (community police in same stations)</t>
         </is>
       </c>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — policing reoriented to harm reduction; no police response-time target and no separate police stations (folded into the 25 district stations)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="46" customHeight="1">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>Police stations</t>
         </is>
       </c>
-      <c r="B31" s="19" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C31" s="21" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E31" s="20" t="inlineStr">
+      <c r="E31" s="22" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
+      <c r="F31" s="21" t="inlineStr">
+        <is>
+          <t>combined into the 25 district stations (no separate police stations)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="46" customHeight="1">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Hospitals</t>
         </is>
       </c>
-      <c r="B32" s="19" t="inlineStr">
+      <c r="B32" s="21" t="inlineStr">
         <is>
           <t>1 Level-1 trauma (1,200 beds) + 6 district (300 beds) + 25 urgent-care</t>
         </is>
       </c>
-      <c r="C32" s="19" t="inlineStr">
+      <c r="C32" s="21" t="inlineStr">
         <is>
           <t>1 per district hub (6) + none solely in civic core (deliberate)</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
         <is>
           <t>1 Level-1 trauma (civic core) + district clinics</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr">
+      <c r="E32" s="21" t="inlineStr">
         <is>
           <t>4 (core + 3 alternating petals); p99 transport &lt;=10 min; N+1 paired capacity</t>
         </is>
       </c>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <t>5 (city centre + 4 quadrant centres) + local stabilisation clinics</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="46" customHeight="1">
-      <c r="A33" s="18" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>Degraded-response (post-disaster) analysis</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>MISSING — no post-earthquake / station-loss response analysis (contrast: Meridian-F and Meridian-S both model it)</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C33" s="21" t="inlineStr">
         <is>
           <t>double failure (district hub + civic core down): 454 s mean mutual aid — stated as accepted limitation; 72 h cell reserves are the fallback</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D33" s="23" t="inlineStr">
         <is>
           <t>MISSING — islandable microgrids and looped utilidors stated for lifelines, but no station-loss response-time analysis</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>25% of stations destroyed: mean 2.6 / p90 3.6 / max 4.9 min — still beats intact 7-station design (computed)</t>
         </is>
       </c>
+      <c r="F33" s="21" t="inlineStr">
+        <is>
+          <t>degraded-road (25 km/h) worst-corner 7.05 min; no emergency facility dependent on one bridge/pipe/substation/data link; &gt;=2 physically separate routes into every district</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>— Crime, economy, society —</t>
         </is>
       </c>
-      <c r="B34" s="17" t="n"/>
-      <c r="C34" s="17" t="n"/>
-      <c r="D34" s="17" t="n"/>
-      <c r="E34" s="17" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
     </row>
     <row r="35" ht="46" customHeight="1">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>Crime target (see metric)</t>
         </is>
       </c>
-      <c r="B35" s="19" t="inlineStr">
+      <c r="B35" s="21" t="inlineStr">
         <is>
           <t>15 crimes per 100k/yr  [total crime/100k]</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C35" s="21" t="inlineStr">
         <is>
           <t>150 violent crimes per 100k/yr  [violent crime/100k]</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>1 homicides per 100k/yr  [homicide/100k]</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>0.5 homicides per 100k/yr  [homicide/100k]</t>
         </is>
       </c>
+      <c r="F35" s="21" t="inlineStr">
+        <is>
+          <t>2 homicides per 100k/yr  [homicide/100k]</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="46" customHeight="1">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>Incarceration target (per 100k)</t>
         </is>
       </c>
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>50 prisoners per 100k</t>
         </is>
       </c>
-      <c r="C36" s="21" t="inlineStr">
+      <c r="C36" s="23" t="inlineStr">
         <is>
           <t>MISSING — restorative-first track stated; no incarceration-rate number</t>
         </is>
       </c>
-      <c r="D36" s="21" t="inlineStr">
+      <c r="D36" s="23" t="inlineStr">
         <is>
           <t>MISSING — incarceration 'last resort'; no rate target</t>
         </is>
       </c>
-      <c r="E36" s="21" t="inlineStr">
+      <c r="E36" s="23" t="inlineStr">
         <is>
           <t>MISSING — custody 'reserved for danger'; Norway ~20% recidivism benchmark; no rate number</t>
         </is>
       </c>
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — prisons 'reserved primarily for continuing serious risk'; no incarceration-rate number</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="46" customHeight="1">
-      <c r="A37" s="18" t="inlineStr">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>Economic model</t>
         </is>
       </c>
-      <c r="B37" s="19" t="inlineStr">
+      <c r="B37" s="21" t="inlineStr">
         <is>
           <t>Hybrid cooperative capitalism</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="C37" s="21" t="inlineStr">
         <is>
           <t>Commons/market hybrid (3 tiers)</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>Stakeholder market on a universal foundation</t>
         </is>
       </c>
-      <c r="E37" s="19" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>Market Georgism with a universal floor</t>
         </is>
       </c>
+      <c r="F37" s="21" t="inlineStr">
+        <is>
+          <t>Constitutional social-market and commons economy</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="46" customHeight="1">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>Gini coefficient target</t>
         </is>
       </c>
-      <c r="B38" s="19" t="inlineStr">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>0.28</t>
         </is>
       </c>
-      <c r="C38" s="21" t="inlineStr">
+      <c r="C38" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="D38" s="21" t="inlineStr">
+      <c r="D38" s="23" t="inlineStr">
         <is>
           <t>MISSING — 'compresses inequality by construction' — no number</t>
         </is>
       </c>
-      <c r="E38" s="21" t="inlineStr">
+      <c r="E38" s="23" t="inlineStr">
         <is>
           <t>MISSING — 'inequality compression' is lever #1 but no Gini number</t>
         </is>
       </c>
+      <c r="F38" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — contentment thresholds set (&gt;=80% life satisfaction, no quintile gap) but no Gini figure</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>— Self-sufficiency —</t>
         </is>
       </c>
-      <c r="B39" s="17" t="n"/>
-      <c r="C39" s="17" t="n"/>
-      <c r="D39" s="17" t="n"/>
-      <c r="E39" s="17" t="n"/>
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
     </row>
     <row r="40" ht="46" customHeight="1">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="20" t="inlineStr">
         <is>
           <t>Energy demand, average (MW)</t>
         </is>
       </c>
-      <c r="B40" s="19" t="inlineStr">
+      <c r="B40" s="21" t="inlineStr">
         <is>
           <t>1200 MW</t>
         </is>
       </c>
-      <c r="C40" s="21" t="inlineStr">
+      <c r="C40" s="23" t="inlineStr">
         <is>
           <t>MISSING — peak stated, average not</t>
         </is>
       </c>
-      <c r="D40" s="19" t="inlineStr">
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>266 MW</t>
         </is>
       </c>
-      <c r="E40" s="19" t="inlineStr">
+      <c r="E40" s="21" t="inlineStr">
         <is>
           <t>630 MW</t>
         </is>
       </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>913 MW</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="46" customHeight="1">
-      <c r="A41" s="18" t="inlineStr">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>Energy demand, peak (MW)</t>
         </is>
       </c>
-      <c r="B41" s="21" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="C41" s="19" t="inlineStr">
+      <c r="C41" s="21" t="inlineStr">
         <is>
           <t>685 MW design peak</t>
         </is>
       </c>
-      <c r="D41" s="19" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>532 MW</t>
         </is>
       </c>
-      <c r="E41" s="19" t="inlineStr">
+      <c r="E41" s="21" t="inlineStr">
         <is>
           <t>1500 MW</t>
         </is>
       </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — no peak load stated; the 2.5 GW figure is an emergency-demand / firm-capability target, not a peak load</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="46" customHeight="1">
-      <c r="A42" s="18" t="inlineStr">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>Energy mix</t>
         </is>
       </c>
-      <c r="B42" s="19" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t>solar: 40%, wind: 35%, geothermal: 15%, hydro: 10% % annual</t>
         </is>
       </c>
-      <c r="C42" s="19" t="inlineStr">
+      <c r="C42" s="21" t="inlineStr">
         <is>
           <t>offshore_wind: 55%, solar: 30%, tidal_wave_biogas: 15% % supply</t>
         </is>
       </c>
-      <c r="D42" s="19" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>solar PV + wind (dual-use farmland) + geothermal/biogas firm; 1.7x overbuild for seasonal storage via green H2</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr">
+      <c r="E42" s="21" t="inlineStr">
         <is>
           <t>rooftop PV ~1 GWp + 25 km2 hinterland agrivoltaics + wind where available + firm block (geothermal, 2 SMRs, or biomass CHP)</t>
         </is>
       </c>
+      <c r="F42" s="21" t="inlineStr">
+        <is>
+          <t>locally selected portfolio: solar, wind, geothermal, hydro, waste biogas, biomass backup, nuclear only if the no-import rule is genuinely met; &gt;=2.5 GW firm; no single plant &gt;15% of firm capacity</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="46" customHeight="1">
-      <c r="A43" s="18" t="inlineStr">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>Battery storage (GWh)</t>
         </is>
       </c>
-      <c r="B43" s="19" t="inlineStr">
+      <c r="B43" s="21" t="inlineStr">
         <is>
           <t>10 GWh</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C43" s="21" t="inlineStr">
         <is>
           <t>3.4 GWh (~8 h average load)</t>
         </is>
       </c>
-      <c r="D43" s="21" t="inlineStr">
+      <c r="D43" s="23" t="inlineStr">
         <is>
           <t>MISSING — batteries + pumped hydro + H2 + biogas named; capacities not</t>
         </is>
       </c>
-      <c r="E43" s="19" t="inlineStr">
+      <c r="E43" s="21" t="inlineStr">
         <is>
           <t>4 GWh + seasonal sand/water thermal pits</t>
         </is>
       </c>
+      <c r="F43" s="23" t="inlineStr">
+        <is>
+          <t>MISSING — explicitly declines a single battery figure: a 72 h / 180 GWh reserve is stated to be 'too large as lithium batteries alone', met instead by batteries + thermal + water + dispatchable generation + hydrogen</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="46" customHeight="1">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>Energy autonomy (days)</t>
         </is>
       </c>
-      <c r="B44" s="19" t="inlineStr">
+      <c r="B44" s="21" t="inlineStr">
         <is>
           <t>21 days</t>
         </is>
       </c>
-      <c r="C44" s="20" t="inlineStr">
+      <c r="C44" s="22" t="inlineStr">
         <is>
           <t>0.33 days (8 h battery)</t>
         </is>
       </c>
-      <c r="D44" s="21" t="inlineStr">
+      <c r="D44" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="E44" s="21" t="inlineStr">
+      <c r="E44" s="23" t="inlineStr">
         <is>
           <t>MISSING — 72 h islanding per district for critical loads stated; whole-city autonomy days not</t>
         </is>
       </c>
+      <c r="F44" s="21" t="inlineStr">
+        <is>
+          <t>3 days</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="46" customHeight="1">
-      <c r="A45" s="18" t="inlineStr">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>Water demand (m³/day)</t>
         </is>
       </c>
-      <c r="B45" s="19" t="inlineStr">
+      <c r="B45" s="21" t="inlineStr">
         <is>
           <t>2500000 m3/day</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C45" s="21" t="inlineStr">
         <is>
           <t>130800 m3/day</t>
         </is>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D45" s="22" t="inlineStr">
         <is>
           <t>33700 m3/day</t>
         </is>
       </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="E45" s="22" t="inlineStr">
         <is>
           <t>128767 m3/day municipal</t>
         </is>
       </c>
+      <c r="F45" s="21" t="inlineStr">
+        <is>
+          <t>150000 m3/day domestic</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="46" customHeight="1">
-      <c r="A46" s="18" t="inlineStr">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>Water sources</t>
         </is>
       </c>
-      <c r="B46" s="19" t="inlineStr">
+      <c r="B46" s="21" t="inlineStr">
         <is>
           <t>rainfall: 60%, desalination: 25%, recycling: 15%</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr">
+      <c r="C46" s="21" t="inlineStr">
         <is>
           <t>rainfall: 59%, recycling: 40%, desalination: 1%</t>
         </is>
       </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>recycling: 85%, rain_and_aquifer: 15% % approx</t>
         </is>
       </c>
-      <c r="E46" s="19" t="inlineStr">
+      <c r="E46" s="21" t="inlineStr">
         <is>
           <t>rooftop catchment (mandated) + wedge reservoirs + 40% potable reuse; desal only for coastal-arid instances</t>
         </is>
       </c>
+      <c r="F46" s="21" t="inlineStr">
+        <is>
+          <t>protected upland catchments, sustainable-yield groundwater, rainwater, reclaimed wastewater, coastal desalination (fallback), seasonal reservoirs &amp; managed aquifer recharge</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="46" customHeight="1">
-      <c r="A47" s="18" t="inlineStr">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>Water reserve (days)</t>
         </is>
       </c>
-      <c r="B47" s="19" t="inlineStr">
+      <c r="B47" s="21" t="inlineStr">
         <is>
           <t>180 days</t>
         </is>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C47" s="23" t="inlineStr">
         <is>
           <t>MISSING — 72 h cell-hub reserves stated for emergencies; no city-level reserve-days figure</t>
         </is>
       </c>
-      <c r="D47" s="21" t="inlineStr">
+      <c r="D47" s="23" t="inlineStr">
         <is>
           <t>MISSING — not reported in source repo</t>
         </is>
       </c>
-      <c r="E47" s="19" t="inlineStr">
+      <c r="E47" s="21" t="inlineStr">
         <is>
           <t>3 days (72 h per district, L14)</t>
         </is>
       </c>
+      <c r="F47" s="21" t="inlineStr">
+        <is>
+          <t>180 days (regional; district storage &gt;=7 days)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="46" customHeight="1">
-      <c r="A48" s="18" t="inlineStr">
+      <c r="A48" s="20" t="inlineStr">
         <is>
           <t>Food self-sufficiency</t>
         </is>
       </c>
-      <c r="B48" s="19" t="inlineStr">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>100% vegetables+protein, 60% grains target stated in §3.2 header, but §3.2 also claims 2.25 Mt/yr grain surplus; iteration 8 found 50% of meat must be imported</t>
         </is>
       </c>
-      <c r="C48" s="19" t="inlineStr">
+      <c r="C48" s="21" t="inlineStr">
         <is>
           <t>life-critical necessities only, explicitly scoped; staples from 388 km2 hinterland at realistic yields; vertical farms greens-only (88.8 ha)</t>
         </is>
       </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>full calories from 217 km2 regenerative farmland (2,500 kcal +30% loss); CEA for perishables only (479 GWh/yr)</t>
         </is>
       </c>
-      <c r="E48" s="19" t="inlineStr">
+      <c r="E48" s="21" t="inlineStr">
         <is>
           <t>98% of calories from ~1,000 km2 hinterland (plant-forward, 800-1,000 m2/person); vertical farms ~2% of calories (200 ha)</t>
         </is>
       </c>
+      <c r="F48" s="21" t="inlineStr">
+        <is>
+          <t>sized to 110% of caloric need (963.6 Tcal/yr for 1M @ 2,400 kcal/day); plant-forward; 4,000 km² hinterland; urban farms for perishables only (not staple calories)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="46" customHeight="1">
-      <c r="A49" s="18" t="inlineStr">
+      <c r="A49" s="20" t="inlineStr">
         <is>
           <t>Food reserve (months)</t>
         </is>
       </c>
-      <c r="B49" s="19" t="inlineStr">
+      <c r="B49" s="21" t="inlineStr">
         <is>
           <t>6 months (extendable to 12)</t>
         </is>
       </c>
-      <c r="C49" s="19" t="inlineStr">
+      <c r="C49" s="21" t="inlineStr">
         <is>
           <t>0.1 months (72 h per cell hub)</t>
         </is>
       </c>
-      <c r="D49" s="21" t="inlineStr">
+      <c r="D49" s="23" t="inlineStr">
         <is>
           <t>MISSING — 'strategic stockpiles' named for high-tech inputs; food reserve duration not stated</t>
         </is>
       </c>
-      <c r="E49" s="19" t="inlineStr">
+      <c r="E49" s="21" t="inlineStr">
         <is>
           <t>18 months staple grain per district</t>
         </is>
       </c>
+      <c r="F49" s="21" t="inlineStr">
+        <is>
+          <t>12 months staple calories (strategic reserve)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A50" s="18" t="inlineStr">
         <is>
           <t>— Quality of life —</t>
         </is>
       </c>
-      <c r="B50" s="17" t="n"/>
-      <c r="C50" s="17" t="n"/>
-      <c r="D50" s="17" t="n"/>
-      <c r="E50" s="17" t="n"/>
+      <c r="B50" s="19" t="n"/>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+      <c r="E50" s="19" t="n"/>
+      <c r="F50" s="19" t="n"/>
     </row>
     <row r="51" ht="46" customHeight="1">
-      <c r="A51" s="18" t="inlineStr">
+      <c r="A51" s="20" t="inlineStr">
         <is>
           <t>Housing floor (m²/person)</t>
         </is>
       </c>
-      <c r="B51" s="19" t="inlineStr">
+      <c r="B51" s="21" t="inlineStr">
         <is>
           <t>30 m2</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
+      <c r="C51" s="21" t="inlineStr">
         <is>
           <t>35 m2</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="D51" s="21" t="inlineStr">
         <is>
           <t>28 m2</t>
         </is>
       </c>
-      <c r="E51" s="19" t="inlineStr">
+      <c r="E51" s="21" t="inlineStr">
         <is>
           <t>35 m2 net + &gt;=2 rooms/household + 2 h direct sun</t>
         </is>
       </c>
+      <c r="F51" s="21" t="inlineStr">
+        <is>
+          <t>35 m2 (35 one adult, 50 two adults, +12 per extra resident)</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="46" customHeight="1">
-      <c r="A52" s="18" t="inlineStr">
+      <c r="A52" s="20" t="inlineStr">
         <is>
           <t>Noise limits</t>
         </is>
       </c>
-      <c r="B52" s="21" t="inlineStr">
+      <c r="B52" s="23" t="inlineStr">
         <is>
           <t>MISSING — 'strict noise codes' asserted, no numbers</t>
         </is>
       </c>
-      <c r="C52" s="19" t="inlineStr">
+      <c r="C52" s="21" t="inlineStr">
         <is>
           <t>&lt;=55 dB facades / &lt;=45 dB courtyards</t>
         </is>
       </c>
-      <c r="D52" s="19" t="inlineStr">
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>&lt;=55 dB day outdoors / &lt;=30 dB indoors night</t>
         </is>
       </c>
-      <c r="E52" s="19" t="inlineStr">
+      <c r="E52" s="21" t="inlineStr">
         <is>
           <t>&lt;=55 dB(A) day / 45 night at every facade; quiet side mandatory</t>
         </is>
       </c>
+      <c r="F52" s="21" t="inlineStr">
+        <is>
+          <t>&lt;=30 dBA bedroom at night; &lt;=45 dBA exterior residential night where feasible</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="46" customHeight="1">
-      <c r="A53" s="18" t="inlineStr">
+      <c r="A53" s="20" t="inlineStr">
         <is>
           <t>Commute / 15-min-city target</t>
         </is>
       </c>
-      <c r="B53" s="19" t="inlineStr">
+      <c r="B53" s="21" t="inlineStr">
         <is>
           <t>median 25 min edge-to-centre transit</t>
         </is>
       </c>
-      <c r="C53" s="19" t="inlineStr">
+      <c r="C53" s="21" t="inlineStr">
         <is>
           <t>&gt;=90% within 15-minute walk/bike/transit of daily needs</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="D53" s="21" t="inlineStr">
         <is>
           <t>15-minute walk for daily life; any cross-city trip &lt;=15 min</t>
         </is>
       </c>
-      <c r="E53" s="19" t="inlineStr">
+      <c r="E53" s="21" t="inlineStr">
         <is>
           <t>median &lt;=22 min door-to-door, p90 &lt;=35 min; 90% within 15-min walk of daily needs</t>
         </is>
       </c>
+      <c r="F53" s="21" t="inlineStr">
+        <is>
+          <t>median &lt;15 min; p90 &lt;25 min; daily-needs trip &lt;10 min for 90%; 100% of homes within 400 m of daily needs or transit</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="46" customHeight="1">
-      <c r="A54" s="18" t="inlineStr">
+      <c r="A54" s="20" t="inlineStr">
         <is>
           <t>Local emergency reserves</t>
         </is>
       </c>
-      <c r="B54" s="21" t="inlineStr">
+      <c r="B54" s="23" t="inlineStr">
         <is>
           <t>MISSING — no per-neighbourhood 72h reserve concept; city-level reserves only</t>
         </is>
       </c>
-      <c r="C54" s="19" t="inlineStr">
+      <c r="C54" s="21" t="inlineStr">
         <is>
           <t>72 hours (water/food/first-aid per cell hub)</t>
         </is>
       </c>
-      <c r="D54" s="21" t="inlineStr">
+      <c r="D54" s="23" t="inlineStr">
         <is>
           <t>MISSING — islandable district microgrids stated for power; water/food local reserve duration not stated</t>
         </is>
       </c>
-      <c r="E54" s="19" t="inlineStr">
+      <c r="E54" s="21" t="inlineStr">
         <is>
           <t>72 hours water per district + 7 d food distribution capacity (L14)</t>
+        </is>
+      </c>
+      <c r="F54" s="21" t="inlineStr">
+        <is>
+          <t>168 hours (7 days district potable water; + 72 h passive survivability)</t>
         </is>
       </c>
     </row>
@@ -2943,7 +3420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2959,784 +3436,988 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Figure</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>Reason recorded in schema</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>Built-up density (people/km²)</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>masterplan gives ring populations and radii but never a built-up density figure</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Street width (m)</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>'strict building separation distances' asserted in §10.1 but no number anywhere</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>Building spacing / block grid</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>no spacing, setback, or block-grid dimension stated — fire-spread modelling for Solaris is low-confidence</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>Gas grid / ignition source</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>post-quake fire ignition source unaddressed (Meridian-F explicitly bans gas; Solaris silent)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>Soft-storey ban</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>not addressed (waterfront buildings deliberately have open lower storeys for tsunami)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>Site elevation / terrain data</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>no ground elevations, drainage capacities, or inundation map — flood simulation is low-confidence and defence-layer-based only</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>Degraded-response (post-disaster) analysis</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>no post-earthquake / station-loss response analysis (contrast: Meridian-F and Meridian-S both model it)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>Energy demand, peak (MW)</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>Noise limits</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>'strict noise codes' asserted, no numbers</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>Local emergency reserves</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>no per-neighbourhood 72h reserve concept; city-level reserves only</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>Street width (m)</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>cell geometry and 180 m inter-district buffers stated; street cross-sections not</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>Gas grid / ignition source</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>Lateral drift capacity (m)</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>Quake survival target (%)</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>no quantified survival target; qualitative performance goals only</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>Tsunami / surge design height (m)</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C18" s="21" t="inlineStr">
         <is>
           <t>refuge storeys 'above the design tsunami height' and high-ground network at +15-20 m stated, but the design wave height itself is never given</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="25" t="inlineStr">
         <is>
           <t>Stormwater drainage</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>buffers include 'drainage swales' (geometry script) but no capacities</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="25" t="inlineStr">
         <is>
           <t>Fire response, tail (min)</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t>model reports median and zero-points-over-300s, not a p95</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="25" t="inlineStr">
         <is>
           <t>Ambulances</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>Police response (min)</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="21" t="inlineStr">
         <is>
           <t>policing legitimacy/accountability specified; response times and station counts are not</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="25" t="inlineStr">
         <is>
           <t>Police stations</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="25" t="inlineStr">
         <is>
           <t>Incarceration target (per 100k)</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C24" s="21" t="inlineStr">
         <is>
           <t>restorative-first track stated; no incarceration-rate number</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="25" t="inlineStr">
         <is>
           <t>Gini coefficient target</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="B26" s="25" t="inlineStr">
         <is>
           <t>Energy demand, average (MW)</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C26" s="21" t="inlineStr">
         <is>
           <t>peak stated, average not</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="24" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B27" s="23" t="inlineStr">
+      <c r="B27" s="25" t="inlineStr">
         <is>
           <t>Water reserve (days)</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C27" s="21" t="inlineStr">
         <is>
           <t>72 h cell-hub reserves stated for emergencies; no city-level reserve-days figure</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="25" t="inlineStr">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B28" s="23" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>Street width (m)</t>
         </is>
       </c>
-      <c r="C28" s="19" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>block typology described; street cross-sections not dimensioned</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="25" t="inlineStr">
+      <c r="A29" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B29" s="23" t="inlineStr">
+      <c r="B29" s="25" t="inlineStr">
         <is>
           <t>Building spacing / block grid</t>
         </is>
       </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>perimeter-block courtyards implied; no block-grid dimension given</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="25" t="inlineStr">
+      <c r="A30" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B30" s="23" t="inlineStr">
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>Gas grid / ignition source</t>
         </is>
       </c>
-      <c r="C30" s="19" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>buried utilities stated for wind; gas not addressed</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="A31" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>Soft-storey ban</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="C31" s="21" t="inlineStr">
         <is>
           <t>strong-column/weak-beam stated; explicit soft-storey prohibition not stated (seaward pilotis blocks are deliberately open-ground)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="25" t="inlineStr">
+      <c r="A32" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B32" s="25" t="inlineStr">
         <is>
           <t>Lateral drift capacity (m)</t>
         </is>
       </c>
-      <c r="C32" s="19" t="inlineStr">
+      <c r="C32" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
+      <c r="A33" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>Quake survival target (%)</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C33" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="25" t="inlineStr">
+      <c r="A34" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B34" s="23" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
         <is>
           <t>Tsunami / surge design height (m)</t>
         </is>
       </c>
-      <c r="C34" s="19" t="inlineStr">
+      <c r="C34" s="21" t="inlineStr">
         <is>
           <t>layered defence + FEMA P-646 refuges stated; design wave height region-tuned, never numbered</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="25" t="inlineStr">
+      <c r="A35" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>Ambulances</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C35" s="21" t="inlineStr">
         <is>
           <t>hubs co-locate EMS; vehicle counts not given</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="25" t="inlineStr">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B36" s="23" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
         <is>
           <t>Degraded-response (post-disaster) analysis</t>
         </is>
       </c>
-      <c r="C36" s="19" t="inlineStr">
+      <c r="C36" s="21" t="inlineStr">
         <is>
           <t>islandable microgrids and looped utilidors stated for lifelines, but no station-loss response-time analysis</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="25" t="inlineStr">
+      <c r="A37" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B37" s="23" t="inlineStr">
+      <c r="B37" s="25" t="inlineStr">
         <is>
           <t>Incarceration target (per 100k)</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="C37" s="21" t="inlineStr">
         <is>
           <t>incarceration 'last resort'; no rate target</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="25" t="inlineStr">
+      <c r="A38" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B38" s="23" t="inlineStr">
+      <c r="B38" s="25" t="inlineStr">
         <is>
           <t>Gini coefficient target</t>
         </is>
       </c>
-      <c r="C38" s="19" t="inlineStr">
+      <c r="C38" s="21" t="inlineStr">
         <is>
           <t>'compresses inequality by construction' — no number</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
+      <c r="A39" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B39" s="23" t="inlineStr">
+      <c r="B39" s="25" t="inlineStr">
         <is>
           <t>Battery storage (GWh)</t>
         </is>
       </c>
-      <c r="C39" s="19" t="inlineStr">
+      <c r="C39" s="21" t="inlineStr">
         <is>
           <t>batteries + pumped hydro + H2 + biogas named; capacities not</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="25" t="inlineStr">
+      <c r="A40" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B40" s="23" t="inlineStr">
+      <c r="B40" s="25" t="inlineStr">
         <is>
           <t>Energy autonomy (days)</t>
         </is>
       </c>
-      <c r="C40" s="19" t="inlineStr">
+      <c r="C40" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
+      <c r="A41" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B41" s="23" t="inlineStr">
+      <c r="B41" s="25" t="inlineStr">
         <is>
           <t>Water reserve (days)</t>
         </is>
       </c>
-      <c r="C41" s="19" t="inlineStr">
+      <c r="C41" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="25" t="inlineStr">
+      <c r="A42" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B42" s="23" t="inlineStr">
+      <c r="B42" s="25" t="inlineStr">
         <is>
           <t>Food reserve (months)</t>
         </is>
       </c>
-      <c r="C42" s="19" t="inlineStr">
+      <c r="C42" s="21" t="inlineStr">
         <is>
           <t>'strategic stockpiles' named for high-tech inputs; food reserve duration not stated</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
+      <c r="A43" s="27" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B43" s="23" t="inlineStr">
+      <c r="B43" s="25" t="inlineStr">
         <is>
           <t>Local emergency reserves</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C43" s="21" t="inlineStr">
         <is>
           <t>islandable district microgrids stated for power; water/food local reserve duration not stated</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="26" t="inlineStr">
+      <c r="A44" s="28" t="inlineStr">
         <is>
           <t>Meridian (Fable)</t>
         </is>
       </c>
-      <c r="B44" s="23" t="inlineStr">
+      <c r="B44" s="25" t="inlineStr">
         <is>
           <t>Lateral drift capacity (m)</t>
         </is>
       </c>
-      <c r="C44" s="19" t="inlineStr">
+      <c r="C44" s="21" t="inlineStr">
         <is>
           <t>not reported</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="26" t="inlineStr">
+      <c r="A45" s="28" t="inlineStr">
         <is>
           <t>Meridian (Fable)</t>
         </is>
       </c>
-      <c r="B45" s="23" t="inlineStr">
+      <c r="B45" s="25" t="inlineStr">
         <is>
           <t>Quake survival target (%)</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C45" s="21" t="inlineStr">
         <is>
           <t>no % survival target; instead a functional target — lattice still serves city with 25% of stations destroyed (computed)</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="26" t="inlineStr">
+      <c r="A46" s="28" t="inlineStr">
         <is>
           <t>Meridian (Fable)</t>
         </is>
       </c>
-      <c r="B46" s="23" t="inlineStr">
+      <c r="B46" s="25" t="inlineStr">
         <is>
           <t>Incarceration target (per 100k)</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr">
+      <c r="C46" s="21" t="inlineStr">
         <is>
           <t>custody 'reserved for danger'; Norway ~20% recidivism benchmark; no rate number</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="26" t="inlineStr">
+      <c r="A47" s="28" t="inlineStr">
         <is>
           <t>Meridian (Fable)</t>
         </is>
       </c>
-      <c r="B47" s="23" t="inlineStr">
+      <c r="B47" s="25" t="inlineStr">
         <is>
           <t>Gini coefficient target</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C47" s="21" t="inlineStr">
         <is>
           <t>'inequality compression' is lever #1 but no Gini number</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="26" t="inlineStr">
+      <c r="A48" s="28" t="inlineStr">
         <is>
           <t>Meridian (Fable)</t>
         </is>
       </c>
-      <c r="B48" s="23" t="inlineStr">
+      <c r="B48" s="25" t="inlineStr">
         <is>
           <t>Energy autonomy (days)</t>
         </is>
       </c>
-      <c r="C48" s="19" t="inlineStr">
+      <c r="C48" s="21" t="inlineStr">
         <is>
           <t>72 h islanding per district for critical loads stated; whole-city autonomy days not</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="inlineStr">
+        <is>
+          <t>Street width (m)</t>
+        </is>
+      </c>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>superblocks + redundant street grid described; no street cross-section dimension stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B50" s="25" t="inlineStr">
+        <is>
+          <t>Building spacing / block grid</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>2×2 km districts with superblocks and a redundant utility/transit street grid stated, but no block-grid dimension — fire-spread geometry approximated</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="inlineStr">
+        <is>
+          <t>Soft-storey ban</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>capacity design + strong-column/weak-beam stated, but no explicit soft-storey prohibition (contrast Meridian-F/S which ban it outright)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B52" s="25" t="inlineStr">
+        <is>
+          <t>Lateral drift capacity (m)</t>
+        </is>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B53" s="25" t="inlineStr">
+        <is>
+          <t>Quake survival target (%)</t>
+        </is>
+      </c>
+      <c r="C53" s="21" t="inlineStr">
+        <is>
+          <t>qualitative 'no collapse at MCE / no progressive collapse beyond design'; no % survival figure</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B54" s="25" t="inlineStr">
+        <is>
+          <t>Tsunami / surge design height (m)</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>defence is avoidance (build landward of the site-specific extreme inundation line); the inundation height itself is never numbered</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="inlineStr">
+        <is>
+          <t>Ambulances</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>combined stations described; ambulance/vehicle counts not given</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B56" s="25" t="inlineStr">
+        <is>
+          <t>Police response (min)</t>
+        </is>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>policing reoriented to harm reduction; no police response-time target and no separate police stations (folded into the 25 district stations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="inlineStr">
+        <is>
+          <t>Incarceration target (per 100k)</t>
+        </is>
+      </c>
+      <c r="C57" s="21" t="inlineStr">
+        <is>
+          <t>prisons 'reserved primarily for continuing serious risk'; no incarceration-rate number</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B58" s="25" t="inlineStr">
+        <is>
+          <t>Gini coefficient target</t>
+        </is>
+      </c>
+      <c r="C58" s="21" t="inlineStr">
+        <is>
+          <t>contentment thresholds set (&gt;=80% life satisfaction, no quintile gap) but no Gini figure</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B59" s="25" t="inlineStr">
+        <is>
+          <t>Energy demand, peak (MW)</t>
+        </is>
+      </c>
+      <c r="C59" s="21" t="inlineStr">
+        <is>
+          <t>no peak load stated; the 2.5 GW figure is an emergency-demand / firm-capability target, not a peak load</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="29" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B60" s="25" t="inlineStr">
+        <is>
+          <t>Battery storage (GWh)</t>
+        </is>
+      </c>
+      <c r="C60" s="21" t="inlineStr">
+        <is>
+          <t>explicitly declines a single battery figure: a 72 h / 180 GWh reserve is stated to be 'too large as lithium batteries alone', met instead by batteries + thermal + water + dispatchable generation + hydrogen</t>
         </is>
       </c>
     </row>
@@ -3754,7 +4435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3769,166 +4450,178 @@
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>Status tags</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr"/>
+      <c r="B3" s="31" t="inlineStr"/>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>(plain)</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>Figure stated explicitly in the source repo (masterplan, script, or data file).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>blue text</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>DERIVED — arithmetic on stated figures; the formula is in the cell comment.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>orange fill 'MISSING'</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
         <is>
           <t>The source repo does NOT report this figure. No value was inferred or invented.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>cell comments</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>Hover a value for its source location, precise definition, and caveats.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="9" t="inlineStr"/>
-      <c r="B8" s="28" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="31" t="inlineStr"/>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Why figures are not directly comparable</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr"/>
+      <c r="B9" s="31" t="inlineStr"/>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Crime targets</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>Different metrics: Solaris = total crime, Meridian-S = violent crime, CIVITAS &amp; Meridian-F = homicide. Never rank on this column.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Response times</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>Different definitions: some are travel-only, some end-to-end (incl. dispatch+turnout). Each cell comment states which.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Density</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="31" t="inlineStr">
         <is>
           <t>Solaris's area includes agricultural rings inside the city boundary; the others exclude hinterland.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="9" t="inlineStr"/>
-      <c r="B13" s="28" t="inlineStr"/>
+      <c r="A13" s="10" t="inlineStr"/>
+      <c r="B13" s="31" t="inlineStr"/>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>Source repos</t>
         </is>
       </c>
-      <c r="B14" s="28" t="inlineStr"/>
+      <c r="B14" s="31" t="inlineStr"/>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>Solaris</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t>claude-code-haiku — concentric rings, 25 km radius, 520k people</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Meridian (Sonnet)</t>
         </is>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t>claude-code-sonnet — fractal hex-of-hexes, 467k people</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="32" t="inlineStr">
         <is>
           <t>CIVITAS</t>
         </is>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>claude-code-opus — single hexagon module, 250k people</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>Meridian (Fable)</t>
         </is>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>claude-code-fable/worldwide-city — hex flower, 1M people</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>Resilient City (ChatGPT)</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>chat-gpt-code/resilient-city — 5x5 square grid of 2 km districts, 1M people (added later; a ChatGPT design, not a Claude-model one)</t>
         </is>
       </c>
     </row>

</xml_diff>